<commit_message>
docs: dien link video §7 + sua so lieu lech va noi dung loi thoi (final pass)
Link video: https://www.youtube.com/watch?v=I8-LSwX6y5s
-> README (bang lien ket), report/main-report.md §10, .claude/skills/demo-video-link.md (moi)

Sua so lieu SAI (da kiem chung lai tu nguon goc):
- README: "141 AI + 20 SV" -> 138 + 20 = 158 (truoc do cong ra 161, khong khop)
- Regression: "110/157 case" / "108/157" -> 112/163 request (dem tu collection that)
- So LOG trong ai-audit: 12 -> 14
- README tro nham luot CI xanh #33363058905 -> #33649674605 (khop ci-report)
- docs/10, docs/15, HUONG-DAN: "20 bug" -> 27 bug

Xoa noi dung da loi thoi:
- main-report: "So do tu ve: CHUA LAM" (da ve xong tu 31/08)
- main-report: "Chua lam: Mock Server, Monitor, data-driven" (ca 3 da xong)
- docs/16: bang self-assessment trong -> tro ve ban da dien trong README
- ai-audit + ROADMAP: cap nhat lai muc "viec con lai"

Excel sinh lai: 158 case (51+57+50), khop specs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/23127183_HW06_TestCases.xlsx
+++ b/excel/23127183_HW06_TestCases.xlsx
@@ -464,7 +464,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>&gt; Sinh luc: 2026-09-02T15:27:57.633Z</t>
+          <t>&gt; Sinh luc: 2026-09-02T17:12:00.823Z</t>
         </is>
       </c>
     </row>
@@ -488,21 +488,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>| api-01-login | 53 | 53 | 44 | 9 | 23127183_api-01-login_20260902-222409.json |</t>
+          <t>| api-01-login | 53 | 53 | 44 | 9 | 23127183_api-01-login_20260903-001136.json |</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>| api-02-apply-coupon | 59 | 59 | 46 | 13 | 23127183_api-02-apply-coupon_20260902-222617.json |</t>
+          <t>| api-02-apply-coupon | 59 | 59 | 46 | 13 | 23127183_api-02-apply-coupon_20260903-001136.json |</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>| api-03-product-update | 51 | 51 | 26 | 25 | 23127183_api-03-product-update_20260902-222733.json |</t>
+          <t>| api-03-product-update | 51 | 51 | 26 | 25 | 23127183_api-03-product-update_20260903-001136.json |</t>
         </is>
       </c>
     </row>

</xml_diff>